<commit_message>
docs: refresh science source materials
</commit_message>
<xml_diff>
--- a/Science-notes-links.xlsx
+++ b/Science-notes-links.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\combined-pdf-tex-scraping-main\combined-pdf-tex-scraping-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A197730-1A31-4FA8-8D5F-0D22302C6E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C04920A-4F60-4E31-B4A8-F7F1520D2167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="2" xr2:uid="{4DF391E6-4D08-40A8-B826-18544862AE5D}"/>
+    <workbookView xWindow="5355" yWindow="4065" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{4DF391E6-4D08-40A8-B826-18544862AE5D}"/>
   </bookViews>
   <sheets>
     <sheet name="Class 8th" sheetId="1" r:id="rId1"/>
@@ -131,19 +131,19 @@
     <t>https://edurev.in/t/366484/Chapter-Notes-Temperature-and-its-Measurement/#course_86858</t>
   </si>
   <si>
-    <t>https://edurev.in/t/366524/Chapter-Notes-A-Journey-through-States-of-Water/#course_86858</t>
-  </si>
-  <si>
-    <t>https://edurev.in/t/366525/Chapter-Notes-Methods-of-Separation-in-Everyday-Life/#course_86858</t>
-  </si>
-  <si>
-    <t>https://edurev.in/t/366526/Chapter-Notes-Living-Creatures-Exploring-their-Characteristics/#course_86858</t>
-  </si>
-  <si>
     <t>https://edurev.in/t/366555/Chapter-Notes-Nature-s-Treasures/#course_86858</t>
   </si>
   <si>
     <t>https://edurev.in/t/366582/Chapter-Notes-Beyond-Earth/#course_86858</t>
+  </si>
+  <si>
+    <t>https://edurev.in/t/366405/Exploring-Magnets-Important-Notes-Class-6-Science#course_86858</t>
+  </si>
+  <si>
+    <t>https://edurev.in/t/366468/Chapter-Notes-Materials-Around-Us/#course_86858</t>
+  </si>
+  <si>
+    <t>https://edurev.in/t/366391/Chapter-Notes-Mindful-Eating-A-Path-to-a-Healthy-Body</t>
   </si>
 </sst>
 </file>
@@ -687,34 +687,34 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -722,7 +722,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -730,7 +730,7 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>